<commit_message>
Configura capa e corrige video intro
</commit_message>
<xml_diff>
--- a/outputs/central-configuracao-krisna-fernando.xlsx
+++ b/outputs/central-configuracao-krisna-fernando.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MENSAGENS" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CONFIG'!$A$1:$C$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CONFIG'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'PAGINAS'!$A$1:$H$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CONVIDADOS'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'RSVP'!$A$1:$G$2</definedName>
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -741,186 +741,186 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>ceremony_date_label</t>
+          <t>hero_image</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>29 de outubro de 2026</t>
+          <t>_BQH1940.jpg</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Texto amigável da data</t>
+          <t>Foto de capa. Use o nome do arquivo da GALERIA, sem a extensão final gerada</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>ceremony_time</t>
+          <t>intro_video</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>15h30</t>
+          <t>assets/video/intro-casal.mp4</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Horário da cerimônia</t>
+          <t>Arquivo de vídeo da intro</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>venue_name</t>
+          <t>ceremony_date_label</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Buffet La Maison</t>
+          <t>29 de outubro de 2026</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Nome do local</t>
+          <t>Texto amigável da data</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>ceremony_room</t>
+          <t>ceremony_time</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Salão Terrasse</t>
+          <t>15h30</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Sala da cerimônia</t>
+          <t>Horário da cerimônia</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>reception_room</t>
+          <t>venue_name</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Salão Central</t>
+          <t>Buffet La Maison</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Sala da recepção</t>
+          <t>Nome do local</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>venue_address</t>
+          <t>ceremony_room</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Av. Eng. Luiz Vieira, 555, Papicu</t>
+          <t>Salão Terrasse</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Endereço</t>
+          <t>Sala da cerimônia</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>maps_url</t>
+          <t>reception_room</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Buffet%20La%20Maison%20Av.%20Eng.%20Luiz%20Vieira%20555%20Papicu</t>
+          <t>Salão Central</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Link de rota</t>
+          <t>Sala da recepção</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>whatsapp_contact</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr"/>
+          <t>venue_address</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Av. Eng. Luiz Vieira, 555, Papicu</t>
+        </is>
+      </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Contato do casal ou assessoria</t>
+          <t>Endereço</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>instagram_url</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr"/>
+          <t>maps_url</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Buffet%20La%20Maison%20Av.%20Eng.%20Luiz%20Vieira%20555%20Papicu</t>
+        </is>
+      </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Instagram opcional</t>
+          <t>Link de rota</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>rsvp_enabled</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>whatsapp_contact</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Ativa/desativa formulário</t>
+          <t>Contato do casal ou assessoria</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>gifts_enabled</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
+          <t>instagram_url</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Ativa/desativa presentes</t>
+          <t>Instagram opcional</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>intro_enabled</t>
+          <t>rsvp_enabled</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -930,29 +930,63 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Ativa/desativa intro em vídeo</t>
+          <t>Ativa/desativa formulário</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>gifts_enabled</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Ativa/desativa presentes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>intro_enabled</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Ativa/desativa intro em vídeo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
           <t>site_status</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>preview</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>preview ou published</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C17"/>
+  <autoFilter ref="A1:C19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Move video para hero e refina loader
</commit_message>
<xml_diff>
--- a/outputs/central-configuracao-krisna-fernando.xlsx
+++ b/outputs/central-configuracao-krisna-fernando.xlsx
@@ -758,7 +758,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>intro_video</t>
+          <t>hero_video</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Arquivo de vídeo da intro</t>
+          <t>Vídeo de fundo do topo/hero</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>intro_enabled</t>
+          <t>hero_video_enabled</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Ativa/desativa intro em vídeo</t>
+          <t>Ativa/desativa vídeo de fundo do topo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona check-in por QR Code
</commit_message>
<xml_diff>
--- a/outputs/central-configuracao-krisna-fernando.xlsx
+++ b/outputs/central-configuracao-krisna-fernando.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCOES" sheetId="1" r:id="R23d5b241428441b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG" sheetId="2" r:id="R540d3821c0924afd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PAGINAS" sheetId="3" r:id="R46435ab984a64cdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONVIDADOS" sheetId="4" r:id="Rbcf6036952a449be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RSVP" sheetId="5" r:id="R3b07bf804cb94321"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRESENTES" sheetId="6" r:id="R06a22d5286d14d06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PEDIDOS_PRESENTES" sheetId="7" r:id="R812fa3af9252401a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GALERIA" sheetId="8" r:id="Rfab836d5c9184bf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MENSAGENS" sheetId="9" r:id="Rd772731adf714d2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCOES" sheetId="1" r:id="R08c34cf697644444"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG" sheetId="2" r:id="R984f1f48a4b14158"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PAGINAS" sheetId="3" r:id="Rd45d981db6dd4ef4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONVIDADOS" sheetId="4" r:id="R3e1df68cd67e4ea7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RSVP" sheetId="5" r:id="Rc1822dfa86a84d6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRESENTES" sheetId="6" r:id="R0d0354544d094423"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PEDIDOS_PRESENTES" sheetId="7" r:id="R4e2fba3d8e9446f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPERADORES" sheetId="8" r:id="R2b2cee5d01434662"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GALERIA" sheetId="9" r:id="Rbd30bcc576404291"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MENSAGENS" sheetId="10" r:id="R0acc4ef3145e477e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -394,71 +395,129 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="8" t="str">
-        <x:v>GALERIA</x:v>
+        <x:v>OPERADORES</x:v>
       </x:c>
       <x:c r="B11" s="8" t="str">
-        <x:v>Fotos que podem ser exibidas no site.</x:v>
+        <x:v>Acessos da equipe para validar QR Codes no dia do evento.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="8" t="str">
+        <x:v>GALERIA</x:v>
+      </x:c>
+      <x:c r="B12" s="8" t="str">
+        <x:v>Fotos que podem ser exibidas no site.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="8" t="str">
         <x:v>MENSAGENS</x:v>
       </x:c>
-      <x:c r="B12" s="8" t="str">
+      <x:c r="B13" s="8" t="str">
         <x:v>Mensagens ou depoimentos opcionais.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="8" t="str"/>
-      <x:c r="B13" s="8" t="str"/>
-    </x:row>
     <x:row r="14">
-      <x:c r="A14" s="8" t="str">
-        <x:v>Publicação do Apps Script</x:v>
-      </x:c>
+      <x:c r="A14" s="8" t="str"/>
       <x:c r="B14" s="8" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="8" t="str">
-        <x:v>1. Extensões &gt; Apps Script</x:v>
+        <x:v>Publicação do Apps Script</x:v>
       </x:c>
       <x:c r="B15" s="8" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="8" t="str">
-        <x:v>2. Cole o conteúdo de appscript/Code.gs</x:v>
+        <x:v>1. Extensões &gt; Apps Script</x:v>
       </x:c>
       <x:c r="B16" s="8" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="8" t="str">
-        <x:v>3. Implantar &gt; Nova implantação &gt; App da Web</x:v>
+        <x:v>2. Cole o conteúdo de appscript/Code.gs</x:v>
       </x:c>
       <x:c r="B17" s="8" t="str"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="8" t="str">
-        <x:v>4. Executar como: Eu</x:v>
+        <x:v>3. Implantar &gt; Nova implantação &gt; App da Web</x:v>
       </x:c>
       <x:c r="B18" s="8" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="8" t="str">
-        <x:v>5. Quem pode acessar: Qualquer pessoa</x:v>
+        <x:v>4. Executar como: Eu</x:v>
       </x:c>
       <x:c r="B19" s="8" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="8" t="str">
+        <x:v>5. Quem pode acessar: Qualquer pessoa</x:v>
+      </x:c>
+      <x:c r="B20" s="8" t="str"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="8" t="str">
         <x:v>6. Copie a URL gerada e cole em js/config.js</x:v>
       </x:c>
-      <x:c r="B20" s="8" t="str"/>
+      <x:c r="B21" s="8" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:B1"/>
     <x:mergeCell ref="A2:B2"/>
   </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="86" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>codigo_mensagem</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>nome</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>mensagem</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>ativo</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>ordem</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="8" t="str">
+        <x:v>M-001</x:v>
+      </x:c>
+      <x:c r="B2" s="8" t="str">
+        <x:v>Krisna &amp; Fernando</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="str">
+        <x:v>Obrigado por fazer parte desse capítulo tão especial da nossa história.</x:v>
+      </x:c>
+      <x:c r="D2" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="E2" s="8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -474,13 +533,13 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>key</x:v>
+        <x:v>chave</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>value</x:v>
+        <x:v>valor</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>description</x:v>
+        <x:v>descricao</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -698,28 +757,28 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>section</x:v>
+        <x:v>secao</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>title</x:v>
+        <x:v>titulo</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>subtitle</x:v>
+        <x:v>subtitulo</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>text</x:v>
+        <x:v>texto</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>button_label</x:v>
+        <x:v>rotulo_botao</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>button_url</x:v>
+        <x:v>link_botao</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>enabled</x:v>
+        <x:v>ativo</x:v>
       </x:c>
       <x:c r="H1" s="6" t="str">
-        <x:v>sort_order</x:v>
+        <x:v>ordem</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -825,7 +884,7 @@
         <x:v>presentes</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>Seu carinho já é parte da nossa casa.</x:v>
+        <x:v>Sua contribuição nos ajuda a começar essa nova etapa.</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
         <x:v>Presentes</x:v>
@@ -883,25 +942,25 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>guest_id</x:v>
+        <x:v>codigo_convidado</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>name</x:v>
+        <x:v>nome</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>phone</x:v>
+        <x:v>telefone</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
         <x:v>email</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>group</x:v>
+        <x:v>grupo</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>allowed_companions</x:v>
+        <x:v>acompanhantes_permitidos</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>notes</x:v>
+        <x:v>observacoes</x:v>
       </x:c>
       <x:c r="H1" s="6" t="str">
         <x:v>status</x:v>
@@ -945,41 +1004,77 @@
     <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="70" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="42" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="34" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="34" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="52" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="52" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="26" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="30" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="34" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="16" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="70" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>timestamp</x:v>
+        <x:v>data_hora</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>guest_id</x:v>
+        <x:v>codigo_convidado</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>guest_name</x:v>
+        <x:v>nome_convidado</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>attendance</x:v>
+        <x:v>presenca</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>companions_confirmed</x:v>
+        <x:v>acompanhantes_confirmados</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>companion_name</x:v>
+        <x:v>nome_acompanhante</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>phone</x:v>
+        <x:v>telefone</x:v>
       </x:c>
       <x:c r="H1" s="6" t="str">
+        <x:v>link_whatsapp</x:v>
+      </x:c>
+      <x:c r="I1" s="6" t="str">
         <x:v>email</x:v>
       </x:c>
-      <x:c r="I1" s="6" t="str">
-        <x:v>source</x:v>
-      </x:c>
       <x:c r="J1" s="6" t="str">
-        <x:v>userAgent</x:v>
+        <x:v>token_checkin</x:v>
+      </x:c>
+      <x:c r="K1" s="6" t="str">
+        <x:v>link_checkin</x:v>
+      </x:c>
+      <x:c r="L1" s="6" t="str">
+        <x:v>qr_code</x:v>
+      </x:c>
+      <x:c r="M1" s="6" t="str">
+        <x:v>status_checkin</x:v>
+      </x:c>
+      <x:c r="N1" s="6" t="str">
+        <x:v>checkin_realizado_em</x:v>
+      </x:c>
+      <x:c r="O1" s="6" t="str">
+        <x:v>checkin_por</x:v>
+      </x:c>
+      <x:c r="P1" s="6" t="str">
+        <x:v>email_confirmacao_enviado_em</x:v>
+      </x:c>
+      <x:c r="Q1" s="6" t="str">
+        <x:v>erro_email_confirmacao</x:v>
+      </x:c>
+      <x:c r="R1" s="6" t="str">
+        <x:v>origem</x:v>
+      </x:c>
+      <x:c r="S1" s="6" t="str">
+        <x:v>navegador</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -993,6 +1088,15 @@
       <x:c r="H2" s="8" t="str"/>
       <x:c r="I2" s="8" t="str"/>
       <x:c r="J2" s="8" t="str"/>
+      <x:c r="K2" s="8" t="str"/>
+      <x:c r="L2" s="8" t="str"/>
+      <x:c r="M2" s="8" t="str"/>
+      <x:c r="N2" s="8" t="str"/>
+      <x:c r="O2" s="8" t="str"/>
+      <x:c r="P2" s="8" t="str"/>
+      <x:c r="Q2" s="8" t="str"/>
+      <x:c r="R2" s="8" t="str"/>
+      <x:c r="S2" s="8" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1014,25 +1118,25 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>gift_id</x:v>
+        <x:v>codigo_presente</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>title</x:v>
+        <x:v>titulo</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>description</x:v>
+        <x:v>descricao</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>image</x:v>
+        <x:v>imagem</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>amount</x:v>
+        <x:v>valor</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>enabled</x:v>
+        <x:v>ativo</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>sort_order</x:v>
+        <x:v>ordem</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -1089,7 +1193,7 @@
         <x:v>Café da manhã dos noivos</x:v>
       </x:c>
       <x:c r="C4" s="8" t="str">
-        <x:v>Para começarmos um dia da lua de mel com carinho e mesa bonita.</x:v>
+        <x:v>Para começarmos um dia da lua de mel com calma e mesa bonita.</x:v>
       </x:c>
       <x:c r="D4" s="8" t="str">
         <x:v>assets/images/gifts/cafe-da-manha.svg</x:v>
@@ -1181,7 +1285,7 @@
         <x:v>Primeiro mercado da casa</x:v>
       </x:c>
       <x:c r="C8" s="8" t="str">
-        <x:v>Aquele empurrão carinhoso para abastecer o novo lar.</x:v>
+        <x:v>Aquela força especial para abastecer o novo lar.</x:v>
       </x:c>
       <x:c r="D8" s="8" t="str">
         <x:v>assets/images/gifts/casa.svg</x:v>
@@ -1431,7 +1535,7 @@
         <x:v>P-018</x:v>
       </x:c>
       <x:c r="B19" s="8" t="str">
-        <x:v>Cota carinho</x:v>
+        <x:v>Contribuição especial</x:v>
       </x:c>
       <x:c r="C19" s="8" t="str">
         <x:v>Um presente simbólico para participar da nossa história do seu jeito.</x:v>
@@ -1478,52 +1582,52 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>created_at</x:v>
+        <x:v>criado_em</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>order_id</x:v>
+        <x:v>codigo_pedido</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>gift_id</x:v>
+        <x:v>codigo_presente</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>gift_title</x:v>
+        <x:v>presente</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>amount</x:v>
+        <x:v>valor</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>giver_name</x:v>
+        <x:v>nome</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>giver_phone</x:v>
+        <x:v>telefone</x:v>
       </x:c>
       <x:c r="H1" s="6" t="str">
-        <x:v>giver_email</x:v>
+        <x:v>email</x:v>
       </x:c>
       <x:c r="I1" s="6" t="str">
-        <x:v>message</x:v>
+        <x:v>mensagem</x:v>
       </x:c>
       <x:c r="J1" s="6" t="str">
         <x:v>status</x:v>
       </x:c>
       <x:c r="K1" s="6" t="str">
-        <x:v>provider</x:v>
+        <x:v>provedor</x:v>
       </x:c>
       <x:c r="L1" s="6" t="str">
-        <x:v>provider_payment_id</x:v>
+        <x:v>codigo_pagamento</x:v>
       </x:c>
       <x:c r="M1" s="6" t="str">
-        <x:v>payment_url</x:v>
+        <x:v>link_pagamento</x:v>
       </x:c>
       <x:c r="N1" s="6" t="str">
-        <x:v>paid_at</x:v>
+        <x:v>pago_em</x:v>
       </x:c>
       <x:c r="O1" s="6" t="str">
-        <x:v>source</x:v>
+        <x:v>origem</x:v>
       </x:c>
       <x:c r="P1" s="6" t="str">
-        <x:v>userAgent</x:v>
+        <x:v>navegador</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -1553,6 +1657,56 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>usuario</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>senha</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>nome</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>ativo</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>observacoes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="8" t="str">
+        <x:v>portaria</x:v>
+      </x:c>
+      <x:c r="B2" s="8" t="str">
+        <x:v>trocar-esta-senha</x:v>
+      </x:c>
+      <x:c r="C2" s="8" t="str">
+        <x:v>Equipe Portaria</x:v>
+      </x:c>
+      <x:c r="D2" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="E2" s="8" t="str">
+        <x:v>Troque a senha antes do evento</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
@@ -1564,25 +1718,25 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>image_id</x:v>
+        <x:v>codigo_imagem</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>file_name</x:v>
+        <x:v>arquivo</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>title</x:v>
+        <x:v>titulo</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>alt_text</x:v>
+        <x:v>texto_alternativo</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>featured</x:v>
+        <x:v>destaque</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
-        <x:v>enabled</x:v>
+        <x:v>ativo</x:v>
       </x:c>
       <x:c r="G1" s="6" t="str">
-        <x:v>sort_order</x:v>
+        <x:v>ordem</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -1675,56 +1829,6 @@
       </x:c>
       <x:c r="G5" s="8" t="n">
         <x:v>4</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="86" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="6" t="str">
-        <x:v>message_id</x:v>
-      </x:c>
-      <x:c r="B1" s="6" t="str">
-        <x:v>name</x:v>
-      </x:c>
-      <x:c r="C1" s="6" t="str">
-        <x:v>message</x:v>
-      </x:c>
-      <x:c r="D1" s="6" t="str">
-        <x:v>enabled</x:v>
-      </x:c>
-      <x:c r="E1" s="6" t="str">
-        <x:v>sort_order</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="8" t="str">
-        <x:v>M-001</x:v>
-      </x:c>
-      <x:c r="B2" s="8" t="str">
-        <x:v>Krisna &amp; Fernando</x:v>
-      </x:c>
-      <x:c r="C2" s="8" t="str">
-        <x:v>Obrigado por fazer parte desse capítulo tão especial da nossa história.</x:v>
-      </x:c>
-      <x:c r="D2" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="E2" s="8" t="n">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Atualiza lista de presentes
</commit_message>
<xml_diff>
--- a/outputs/central-configuracao-krisna-fernando.xlsx
+++ b/outputs/central-configuracao-krisna-fernando.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCOES" sheetId="1" r:id="R08c34cf697644444"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG" sheetId="2" r:id="R984f1f48a4b14158"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PAGINAS" sheetId="3" r:id="Rd45d981db6dd4ef4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONVIDADOS" sheetId="4" r:id="R3e1df68cd67e4ea7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RSVP" sheetId="5" r:id="Rc1822dfa86a84d6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRESENTES" sheetId="6" r:id="R0d0354544d094423"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PEDIDOS_PRESENTES" sheetId="7" r:id="R4e2fba3d8e9446f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPERADORES" sheetId="8" r:id="R2b2cee5d01434662"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GALERIA" sheetId="9" r:id="Rbd30bcc576404291"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MENSAGENS" sheetId="10" r:id="R0acc4ef3145e477e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCOES" sheetId="1" r:id="Rbc0110c20c604b17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG" sheetId="2" r:id="R647e1d8262e64b1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PAGINAS" sheetId="3" r:id="Rc9958a590360474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONVIDADOS" sheetId="4" r:id="R86f1df8c91374f3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RSVP" sheetId="5" r:id="R581d45a955814b32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRESENTES" sheetId="6" r:id="R918d95be99f5473c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PEDIDOS_PRESENTES" sheetId="7" r:id="Rdc404f20bb254650"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPERADORES" sheetId="8" r:id="R2dc3fad0f1ba4e28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GALERIA" sheetId="9" r:id="R6e240e48cafc4d5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MENSAGENS" sheetId="10" r:id="R58dee18e35bf40bd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1144,16 +1144,16 @@
         <x:v>P-001</x:v>
       </x:c>
       <x:c r="B2" s="8" t="str">
-        <x:v>Jantar romântico</x:v>
+        <x:v>Petiscos Gourmet da Tereza</x:v>
       </x:c>
       <x:c r="C2" s="8" t="str">
-        <x:v>Uma noite especial para celebrarmos com calma depois do grande dia.</x:v>
+        <x:v>Porque a verdadeira dona da casa também merece participar.</x:v>
       </x:c>
       <x:c r="D2" s="8" t="str">
-        <x:v>assets/images/gifts/jantar-romantico.svg</x:v>
+        <x:v>assets/images/gifts/custom/1.jpeg</x:v>
       </x:c>
       <x:c r="E2" s="8" t="n">
-        <x:v>250</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="F2" s="8" t="str">
         <x:v>TRUE</x:v>
@@ -1167,13 +1167,13 @@
         <x:v>P-002</x:v>
       </x:c>
       <x:c r="B3" s="8" t="str">
-        <x:v>Cota lua de mel</x:v>
+        <x:v>Afinação Matrimonial</x:v>
       </x:c>
       <x:c r="C3" s="8" t="str">
-        <x:v>Um pedacinho da nossa primeira viagem como marido e esposa.</x:v>
+        <x:v>Contribuição para manter a sanfona afinada e o casamento também.</x:v>
       </x:c>
       <x:c r="D3" s="8" t="str">
-        <x:v>assets/images/gifts/lua-de-mel.svg</x:v>
+        <x:v>assets/images/gifts/custom/2.jpeg</x:v>
       </x:c>
       <x:c r="E3" s="8" t="n">
         <x:v>300</x:v>
@@ -1190,16 +1190,16 @@
         <x:v>P-003</x:v>
       </x:c>
       <x:c r="B4" s="8" t="str">
-        <x:v>Café da manhã dos noivos</x:v>
+        <x:v>Aulas de Paciência para Conviver com um Artista</x:v>
       </x:c>
       <x:c r="C4" s="8" t="str">
-        <x:v>Para começarmos um dia da lua de mel com calma e mesa bonita.</x:v>
+        <x:v>Investimento contínuo.</x:v>
       </x:c>
       <x:c r="D4" s="8" t="str">
-        <x:v>assets/images/gifts/cafe-da-manha.svg</x:v>
+        <x:v>assets/images/gifts/custom/3.jpeg</x:v>
       </x:c>
       <x:c r="E4" s="8" t="n">
-        <x:v>180</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="F4" s="8" t="str">
         <x:v>TRUE</x:v>
@@ -1213,13 +1213,13 @@
         <x:v>P-004</x:v>
       </x:c>
       <x:c r="B5" s="8" t="str">
-        <x:v>Noite de hospedagem</x:v>
+        <x:v>Passagem para a Tereza também curtir a lua de mel</x:v>
       </x:c>
       <x:c r="C5" s="8" t="str">
-        <x:v>Uma diária simbólica para descansarmos depois de tanta emoção.</x:v>
+        <x:v>Para ela entrar no clima da viagem junto com os noivos.</x:v>
       </x:c>
       <x:c r="D5" s="8" t="str">
-        <x:v>assets/images/gifts/hospedagem.svg</x:v>
+        <x:v>assets/images/gifts/custom/4.jpeg</x:v>
       </x:c>
       <x:c r="E5" s="8" t="n">
         <x:v>450</x:v>
@@ -1236,16 +1236,16 @@
         <x:v>P-005</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>Passeio especial</x:v>
+        <x:v>Fundo para manter o estoque de whey e creatina do noivo</x:v>
       </x:c>
       <x:c r="C6" s="8" t="str">
-        <x:v>Uma experiência para guardarmos na memória da nossa viagem.</x:v>
+        <x:v>Não é porque casou que vai sair de forma.</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
-        <x:v>assets/images/gifts/passeio.svg</x:v>
+        <x:v>assets/images/gifts/custom/5.jpeg</x:v>
       </x:c>
       <x:c r="E6" s="8" t="n">
-        <x:v>220</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="F6" s="8" t="str">
         <x:v>TRUE</x:v>
@@ -1259,16 +1259,16 @@
         <x:v>P-006</x:v>
       </x:c>
       <x:c r="B7" s="8" t="str">
-        <x:v>Brinde dos noivos</x:v>
+        <x:v>Mini sanfona pro futuro Fernando Júnior</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
-        <x:v>Uma taça levantada para agradecer por esse novo capítulo.</x:v>
+        <x:v>Primeiro investimento musical da próxima geração.</x:v>
       </x:c>
       <x:c r="D7" s="8" t="str">
-        <x:v>assets/images/gifts/brinde.svg</x:v>
+        <x:v>assets/images/gifts/custom/6.jpeg</x:v>
       </x:c>
       <x:c r="E7" s="8" t="n">
-        <x:v>160</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="F7" s="8" t="str">
         <x:v>TRUE</x:v>
@@ -1282,16 +1282,16 @@
         <x:v>P-007</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>Primeiro mercado da casa</x:v>
+        <x:v>Um Dia de Lua de Mel Sem Pensar em Boletos</x:v>
       </x:c>
       <x:c r="C8" s="8" t="str">
-        <x:v>Aquela força especial para abastecer o novo lar.</x:v>
+        <x:v>Sonho patrocinado.</x:v>
       </x:c>
       <x:c r="D8" s="8" t="str">
-        <x:v>assets/images/gifts/casa.svg</x:v>
+        <x:v>assets/images/gifts/custom/7.jpeg</x:v>
       </x:c>
       <x:c r="E8" s="8" t="n">
-        <x:v>350</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="F8" s="8" t="str">
         <x:v>TRUE</x:v>
@@ -1305,16 +1305,16 @@
         <x:v>P-008</x:v>
       </x:c>
       <x:c r="B9" s="8" t="str">
-        <x:v>Kit cozinha feliz</x:v>
+        <x:v>Milhas para conseguir ter uma lua de mel em 2027</x:v>
       </x:c>
       <x:c r="C9" s="8" t="str">
-        <x:v>Para receitas, cafés, conversas e pequenas alegrias do dia a dia.</x:v>
+        <x:v>Ajude os noivos a decolarem nessa próxima aventura.</x:v>
       </x:c>
       <x:c r="D9" s="8" t="str">
-        <x:v>assets/images/gifts/cozinha.svg</x:v>
+        <x:v>assets/images/gifts/custom/8.jpeg</x:v>
       </x:c>
       <x:c r="E9" s="8" t="n">
-        <x:v>280</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="F9" s="8" t="str">
         <x:v>TRUE</x:v>
@@ -1328,16 +1328,16 @@
         <x:v>P-009</x:v>
       </x:c>
       <x:c r="B10" s="8" t="str">
-        <x:v>Mesa posta</x:v>
+        <x:v>Compensação por Horas de Plantão Perdidas Planejando Casamento</x:v>
       </x:c>
       <x:c r="C10" s="8" t="str">
-        <x:v>Um detalhe bonito para receber amigos e família com amor.</x:v>
+        <x:v>Investimento na terapia.</x:v>
       </x:c>
       <x:c r="D10" s="8" t="str">
-        <x:v>assets/images/gifts/mesa-posta.svg</x:v>
+        <x:v>assets/images/gifts/custom/9.jpeg</x:v>
       </x:c>
       <x:c r="E10" s="8" t="n">
-        <x:v>240</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="F10" s="8" t="str">
         <x:v>TRUE</x:v>
@@ -1351,16 +1351,16 @@
         <x:v>P-010</x:v>
       </x:c>
       <x:c r="B11" s="8" t="str">
-        <x:v>Cantinho do café</x:v>
+        <x:v>Ajude em uma mesa de jantar 8 lugares pra você jantar conosco</x:v>
       </x:c>
       <x:c r="C11" s="8" t="str">
-        <x:v>Para nossos cafés de manhã, de tarde e de depois do almoço.</x:v>
+        <x:v>Um convite antecipado para muitos encontros no novo lar.</x:v>
       </x:c>
       <x:c r="D11" s="8" t="str">
-        <x:v>assets/images/gifts/cafe.svg</x:v>
+        <x:v>assets/images/gifts/custom/10.jpeg</x:v>
       </x:c>
       <x:c r="E11" s="8" t="n">
-        <x:v>320</x:v>
+        <x:v>5000</x:v>
       </x:c>
       <x:c r="F11" s="8" t="str">
         <x:v>TRUE</x:v>
@@ -1374,183 +1374,22 @@
         <x:v>P-011</x:v>
       </x:c>
       <x:c r="B12" s="8" t="str">
-        <x:v>Enxoval dos sonhos</x:v>
+        <x:v>Mostre o quanto você é fã do noivo e invista na carreira dele</x:v>
       </x:c>
       <x:c r="C12" s="8" t="str">
-        <x:v>Lençóis, toalhas e conforto para a rotina ficar mais leve.</x:v>
+        <x:v>Para a noiva não precisar mais pegar plantão.</x:v>
       </x:c>
       <x:c r="D12" s="8" t="str">
-        <x:v>assets/images/gifts/enxoval.svg</x:v>
+        <x:v>assets/images/gifts/custom/11.jpeg</x:v>
       </x:c>
       <x:c r="E12" s="8" t="n">
-        <x:v>400</x:v>
+        <x:v>10000</x:v>
       </x:c>
       <x:c r="F12" s="8" t="str">
         <x:v>TRUE</x:v>
       </x:c>
       <x:c r="G12" s="8" t="n">
         <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="8" t="str">
-        <x:v>P-012</x:v>
-      </x:c>
-      <x:c r="B13" s="8" t="str">
-        <x:v>Tete também casa</x:v>
-      </x:c>
-      <x:c r="C13" s="8" t="str">
-        <x:v>Um mimo simbólico para nossa pequena participar desse momento.</x:v>
-      </x:c>
-      <x:c r="D13" s="8" t="str">
-        <x:v>assets/images/gifts/tete.svg</x:v>
-      </x:c>
-      <x:c r="E13" s="8" t="n">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="F13" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G13" s="8" t="n">
-        <x:v>12</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="8" t="str">
-        <x:v>P-013</x:v>
-      </x:c>
-      <x:c r="B14" s="8" t="str">
-        <x:v>Domingo preguiçoso</x:v>
-      </x:c>
-      <x:c r="C14" s="8" t="str">
-        <x:v>Delivery, filme e descanso para depois da maratona do casamento.</x:v>
-      </x:c>
-      <x:c r="D14" s="8" t="str">
-        <x:v>assets/images/gifts/domingo.svg</x:v>
-      </x:c>
-      <x:c r="E14" s="8" t="n">
-        <x:v>190</x:v>
-      </x:c>
-      <x:c r="F14" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G14" s="8" t="n">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="8" t="str">
-        <x:v>P-014</x:v>
-      </x:c>
-      <x:c r="B15" s="8" t="str">
-        <x:v>Álbum de memórias</x:v>
-      </x:c>
-      <x:c r="C15" s="8" t="str">
-        <x:v>Para eternizar fotos e detalhes desse tempo tão especial.</x:v>
-      </x:c>
-      <x:c r="D15" s="8" t="str">
-        <x:v>assets/images/gifts/memorias.svg</x:v>
-      </x:c>
-      <x:c r="E15" s="8" t="n">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="F15" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G15" s="8" t="n">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="8" t="str">
-        <x:v>P-015</x:v>
-      </x:c>
-      <x:c r="B16" s="8" t="str">
-        <x:v>Flores para a casa</x:v>
-      </x:c>
-      <x:c r="C16" s="8" t="str">
-        <x:v>Um toque de beleza para o começo da nossa vida juntos.</x:v>
-      </x:c>
-      <x:c r="D16" s="8" t="str">
-        <x:v>assets/images/gifts/flores.svg</x:v>
-      </x:c>
-      <x:c r="E16" s="8" t="n">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="F16" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G16" s="8" t="n">
-        <x:v>15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="8" t="str">
-        <x:v>P-016</x:v>
-      </x:c>
-      <x:c r="B17" s="8" t="str">
-        <x:v>Ajuda para o novo lar</x:v>
-      </x:c>
-      <x:c r="C17" s="8" t="str">
-        <x:v>Uma contribuição livre, prática e cheia de significado.</x:v>
-      </x:c>
-      <x:c r="D17" s="8" t="str">
-        <x:v>assets/images/gifts/novo-lar.svg</x:v>
-      </x:c>
-      <x:c r="E17" s="8" t="n">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="F17" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G17" s="8" t="n">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="8" t="str">
-        <x:v>P-017</x:v>
-      </x:c>
-      <x:c r="B18" s="8" t="str">
-        <x:v>Experiência gastronômica</x:v>
-      </x:c>
-      <x:c r="C18" s="8" t="str">
-        <x:v>Um almoço ou jantar para celebrarmos sem pressa.</x:v>
-      </x:c>
-      <x:c r="D18" s="8" t="str">
-        <x:v>assets/images/gifts/experiencia.svg</x:v>
-      </x:c>
-      <x:c r="E18" s="8" t="n">
-        <x:v>380</x:v>
-      </x:c>
-      <x:c r="F18" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G18" s="8" t="n">
-        <x:v>17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="8" t="str">
-        <x:v>P-018</x:v>
-      </x:c>
-      <x:c r="B19" s="8" t="str">
-        <x:v>Contribuição especial</x:v>
-      </x:c>
-      <x:c r="C19" s="8" t="str">
-        <x:v>Um presente simbólico para participar da nossa história do seu jeito.</x:v>
-      </x:c>
-      <x:c r="D19" s="8" t="str">
-        <x:v>assets/images/gifts/presente.svg</x:v>
-      </x:c>
-      <x:c r="E19" s="8" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="F19" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G19" s="8" t="n">
-        <x:v>18</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Melhora enquadramento dos presentes
</commit_message>
<xml_diff>
--- a/outputs/central-configuracao-krisna-fernando.xlsx
+++ b/outputs/central-configuracao-krisna-fernando.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCOES" sheetId="1" r:id="Rbc0110c20c604b17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG" sheetId="2" r:id="R647e1d8262e64b1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PAGINAS" sheetId="3" r:id="Rc9958a590360474b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONVIDADOS" sheetId="4" r:id="R86f1df8c91374f3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RSVP" sheetId="5" r:id="R581d45a955814b32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRESENTES" sheetId="6" r:id="R918d95be99f5473c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PEDIDOS_PRESENTES" sheetId="7" r:id="Rdc404f20bb254650"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPERADORES" sheetId="8" r:id="R2dc3fad0f1ba4e28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GALERIA" sheetId="9" r:id="R6e240e48cafc4d5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MENSAGENS" sheetId="10" r:id="R58dee18e35bf40bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCOES" sheetId="1" r:id="Ra87a00c6ca6345ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG" sheetId="2" r:id="R8db50634612e4abe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PAGINAS" sheetId="3" r:id="Rd7e209b9e1254798"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONVIDADOS" sheetId="4" r:id="Re423d244c5c8466f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RSVP" sheetId="5" r:id="R82e9e228821f46db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRESENTES" sheetId="6" r:id="R5829f4e2d7904971"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PEDIDOS_PRESENTES" sheetId="7" r:id="R72e63ba0d1304c01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPERADORES" sheetId="8" r:id="R5cc1d9c5836b4ff2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GALERIA" sheetId="9" r:id="Rdfbb6c55610343b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MENSAGENS" sheetId="10" r:id="R90f1f800f1604be4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1111,9 +1111,10 @@
     <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="68" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="44" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1130,12 +1131,15 @@
         <x:v>imagem</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
+        <x:v>posicao_imagem</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
         <x:v>valor</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="G1" s="6" t="str">
         <x:v>ativo</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="H1" s="6" t="str">
         <x:v>ordem</x:v>
       </x:c>
     </x:row>
@@ -1152,13 +1156,16 @@
       <x:c r="D2" s="8" t="str">
         <x:v>assets/images/gifts/custom/1.jpeg</x:v>
       </x:c>
-      <x:c r="E2" s="8" t="n">
+      <x:c r="E2" s="8" t="str">
+        <x:v>52% 58%</x:v>
+      </x:c>
+      <x:c r="F2" s="8" t="n">
         <x:v>280</x:v>
       </x:c>
-      <x:c r="F2" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G2" s="8" t="n">
+      <x:c r="G2" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="H2" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -1175,13 +1182,16 @@
       <x:c r="D3" s="8" t="str">
         <x:v>assets/images/gifts/custom/2.jpeg</x:v>
       </x:c>
-      <x:c r="E3" s="8" t="n">
+      <x:c r="E3" s="8" t="str">
+        <x:v>50% 42%</x:v>
+      </x:c>
+      <x:c r="F3" s="8" t="n">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="F3" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G3" s="8" t="n">
+      <x:c r="G3" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="H3" s="8" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -1198,13 +1208,16 @@
       <x:c r="D4" s="8" t="str">
         <x:v>assets/images/gifts/custom/3.jpeg</x:v>
       </x:c>
-      <x:c r="E4" s="8" t="n">
+      <x:c r="E4" s="8" t="str">
+        <x:v>50% 36%</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="n">
         <x:v>400</x:v>
       </x:c>
-      <x:c r="F4" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G4" s="8" t="n">
+      <x:c r="G4" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="H4" s="8" t="n">
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -1221,13 +1234,16 @@
       <x:c r="D5" s="8" t="str">
         <x:v>assets/images/gifts/custom/4.jpeg</x:v>
       </x:c>
-      <x:c r="E5" s="8" t="n">
+      <x:c r="E5" s="8" t="str">
+        <x:v>50% 48%</x:v>
+      </x:c>
+      <x:c r="F5" s="8" t="n">
         <x:v>450</x:v>
       </x:c>
-      <x:c r="F5" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G5" s="8" t="n">
+      <x:c r="G5" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="H5" s="8" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
@@ -1244,13 +1260,16 @@
       <x:c r="D6" s="8" t="str">
         <x:v>assets/images/gifts/custom/5.jpeg</x:v>
       </x:c>
-      <x:c r="E6" s="8" t="n">
+      <x:c r="E6" s="8" t="str">
+        <x:v>50% 40%</x:v>
+      </x:c>
+      <x:c r="F6" s="8" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="F6" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G6" s="8" t="n">
+      <x:c r="G6" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="H6" s="8" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -1267,13 +1286,16 @@
       <x:c r="D7" s="8" t="str">
         <x:v>assets/images/gifts/custom/6.jpeg</x:v>
       </x:c>
-      <x:c r="E7" s="8" t="n">
+      <x:c r="E7" s="8" t="str">
+        <x:v>50% 0%</x:v>
+      </x:c>
+      <x:c r="F7" s="8" t="n">
         <x:v>600</x:v>
       </x:c>
-      <x:c r="F7" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G7" s="8" t="n">
+      <x:c r="G7" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="H7" s="8" t="n">
         <x:v>6</x:v>
       </x:c>
     </x:row>
@@ -1290,13 +1312,16 @@
       <x:c r="D8" s="8" t="str">
         <x:v>assets/images/gifts/custom/7.jpeg</x:v>
       </x:c>
-      <x:c r="E8" s="8" t="n">
+      <x:c r="E8" s="8" t="str">
+        <x:v>50% 48%</x:v>
+      </x:c>
+      <x:c r="F8" s="8" t="n">
         <x:v>700</x:v>
       </x:c>
-      <x:c r="F8" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G8" s="8" t="n">
+      <x:c r="G8" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="H8" s="8" t="n">
         <x:v>7</x:v>
       </x:c>
     </x:row>
@@ -1313,13 +1338,16 @@
       <x:c r="D9" s="8" t="str">
         <x:v>assets/images/gifts/custom/8.jpeg</x:v>
       </x:c>
-      <x:c r="E9" s="8" t="n">
+      <x:c r="E9" s="8" t="str">
+        <x:v>50% 44%</x:v>
+      </x:c>
+      <x:c r="F9" s="8" t="n">
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="F9" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G9" s="8" t="n">
+      <x:c r="G9" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="H9" s="8" t="n">
         <x:v>8</x:v>
       </x:c>
     </x:row>
@@ -1336,13 +1364,16 @@
       <x:c r="D10" s="8" t="str">
         <x:v>assets/images/gifts/custom/9.jpeg</x:v>
       </x:c>
-      <x:c r="E10" s="8" t="n">
+      <x:c r="E10" s="8" t="str">
+        <x:v>50% 38%</x:v>
+      </x:c>
+      <x:c r="F10" s="8" t="n">
         <x:v>2000</x:v>
       </x:c>
-      <x:c r="F10" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G10" s="8" t="n">
+      <x:c r="G10" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="H10" s="8" t="n">
         <x:v>9</x:v>
       </x:c>
     </x:row>
@@ -1359,13 +1390,16 @@
       <x:c r="D11" s="8" t="str">
         <x:v>assets/images/gifts/custom/10.jpeg</x:v>
       </x:c>
-      <x:c r="E11" s="8" t="n">
+      <x:c r="E11" s="8" t="str">
+        <x:v>50% 46%</x:v>
+      </x:c>
+      <x:c r="F11" s="8" t="n">
         <x:v>5000</x:v>
       </x:c>
-      <x:c r="F11" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G11" s="8" t="n">
+      <x:c r="G11" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="H11" s="8" t="n">
         <x:v>10</x:v>
       </x:c>
     </x:row>
@@ -1382,13 +1416,16 @@
       <x:c r="D12" s="8" t="str">
         <x:v>assets/images/gifts/custom/11.jpeg</x:v>
       </x:c>
-      <x:c r="E12" s="8" t="n">
+      <x:c r="E12" s="8" t="str">
+        <x:v>50% 50%</x:v>
+      </x:c>
+      <x:c r="F12" s="8" t="n">
         <x:v>10000</x:v>
       </x:c>
-      <x:c r="F12" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="G12" s="8" t="n">
+      <x:c r="G12" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="H12" s="8" t="n">
         <x:v>11</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Adiciona links PagBank aos presentes
</commit_message>
<xml_diff>
--- a/outputs/central-configuracao-krisna-fernando.xlsx
+++ b/outputs/central-configuracao-krisna-fernando.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCOES" sheetId="1" r:id="Ra87a00c6ca6345ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG" sheetId="2" r:id="R8db50634612e4abe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PAGINAS" sheetId="3" r:id="Rd7e209b9e1254798"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONVIDADOS" sheetId="4" r:id="Re423d244c5c8466f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RSVP" sheetId="5" r:id="R82e9e228821f46db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRESENTES" sheetId="6" r:id="R5829f4e2d7904971"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PEDIDOS_PRESENTES" sheetId="7" r:id="R72e63ba0d1304c01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPERADORES" sheetId="8" r:id="R5cc1d9c5836b4ff2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GALERIA" sheetId="9" r:id="Rdfbb6c55610343b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MENSAGENS" sheetId="10" r:id="R90f1f800f1604be4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCOES" sheetId="1" r:id="R4a10cda6d46a4f86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG" sheetId="2" r:id="R6f874b5435f8402c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PAGINAS" sheetId="3" r:id="R66a477f38ab14936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONVIDADOS" sheetId="4" r:id="R15464e54d7a847d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RSVP" sheetId="5" r:id="Rd40f25083d554840"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRESENTES" sheetId="6" r:id="Ra9cfcba7efc6473b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PEDIDOS_PRESENTES" sheetId="7" r:id="Rdb78848ffeb64404"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPERADORES" sheetId="8" r:id="R141632f65aed49f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GALERIA" sheetId="9" r:id="R199e66d9791a4b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MENSAGENS" sheetId="10" r:id="Rb941374f53b944f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1112,9 +1112,10 @@
     <x:col min="3" max="3" width="68" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="44" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1134,12 +1135,15 @@
         <x:v>posicao_imagem</x:v>
       </x:c>
       <x:c r="F1" s="6" t="str">
+        <x:v>link_pagamento</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
         <x:v>valor</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="H1" s="6" t="str">
         <x:v>ativo</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="str">
+      <x:c r="I1" s="6" t="str">
         <x:v>ordem</x:v>
       </x:c>
     </x:row>
@@ -1159,13 +1163,16 @@
       <x:c r="E2" s="8" t="str">
         <x:v>52% 58%</x:v>
       </x:c>
-      <x:c r="F2" s="8" t="n">
+      <x:c r="F2" s="8" t="str">
+        <x:v>https://pag.ae/81ZoZxg7K</x:v>
+      </x:c>
+      <x:c r="G2" s="8" t="n">
         <x:v>280</x:v>
       </x:c>
-      <x:c r="G2" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="H2" s="8" t="n">
+      <x:c r="H2" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="I2" s="8" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -1185,13 +1192,16 @@
       <x:c r="E3" s="8" t="str">
         <x:v>50% 42%</x:v>
       </x:c>
-      <x:c r="F3" s="8" t="n">
+      <x:c r="F3" s="8" t="str">
+        <x:v>https://pag.ae/81Zo-ipHN</x:v>
+      </x:c>
+      <x:c r="G3" s="8" t="n">
         <x:v>300</x:v>
       </x:c>
-      <x:c r="G3" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="H3" s="8" t="n">
+      <x:c r="H3" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="I3" s="8" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -1211,13 +1221,16 @@
       <x:c r="E4" s="8" t="str">
         <x:v>50% 36%</x:v>
       </x:c>
-      <x:c r="F4" s="8" t="n">
+      <x:c r="F4" s="8" t="str">
+        <x:v>https://pag.ae/81Zo-R6cN</x:v>
+      </x:c>
+      <x:c r="G4" s="8" t="n">
         <x:v>400</x:v>
       </x:c>
-      <x:c r="G4" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="H4" s="8" t="n">
+      <x:c r="H4" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="I4" s="8" t="n">
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -1237,13 +1250,16 @@
       <x:c r="E5" s="8" t="str">
         <x:v>50% 48%</x:v>
       </x:c>
-      <x:c r="F5" s="8" t="n">
+      <x:c r="F5" s="8" t="str">
+        <x:v>https://pag.ae/81Zo_LicK</x:v>
+      </x:c>
+      <x:c r="G5" s="8" t="n">
         <x:v>450</x:v>
       </x:c>
-      <x:c r="G5" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="H5" s="8" t="n">
+      <x:c r="H5" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="I5" s="8" t="n">
         <x:v>4</x:v>
       </x:c>
     </x:row>
@@ -1263,13 +1279,16 @@
       <x:c r="E6" s="8" t="str">
         <x:v>50% 40%</x:v>
       </x:c>
-      <x:c r="F6" s="8" t="n">
+      <x:c r="F6" s="8" t="str">
+        <x:v>https://pag.ae/81Zp1wGVs</x:v>
+      </x:c>
+      <x:c r="G6" s="8" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="G6" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="H6" s="8" t="n">
+      <x:c r="H6" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="I6" s="8" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -1289,13 +1308,16 @@
       <x:c r="E7" s="8" t="str">
         <x:v>50% 0%</x:v>
       </x:c>
-      <x:c r="F7" s="8" t="n">
+      <x:c r="F7" s="8" t="str">
+        <x:v>https://pag.ae/81Zp1Zyzs</x:v>
+      </x:c>
+      <x:c r="G7" s="8" t="n">
         <x:v>600</x:v>
       </x:c>
-      <x:c r="G7" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="H7" s="8" t="n">
+      <x:c r="H7" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="I7" s="8" t="n">
         <x:v>6</x:v>
       </x:c>
     </x:row>
@@ -1315,13 +1337,16 @@
       <x:c r="E8" s="8" t="str">
         <x:v>50% 48%</x:v>
       </x:c>
-      <x:c r="F8" s="8" t="n">
+      <x:c r="F8" s="8" t="str">
+        <x:v>https://pag.ae/81Zp2eM64</x:v>
+      </x:c>
+      <x:c r="G8" s="8" t="n">
         <x:v>700</x:v>
       </x:c>
-      <x:c r="G8" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="H8" s="8" t="n">
+      <x:c r="H8" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="I8" s="8" t="n">
         <x:v>7</x:v>
       </x:c>
     </x:row>
@@ -1341,13 +1366,16 @@
       <x:c r="E9" s="8" t="str">
         <x:v>50% 44%</x:v>
       </x:c>
-      <x:c r="F9" s="8" t="n">
+      <x:c r="F9" s="8" t="str">
+        <x:v>https://pag.ae/81Zp2zXNK</x:v>
+      </x:c>
+      <x:c r="G9" s="8" t="n">
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="G9" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="H9" s="8" t="n">
+      <x:c r="H9" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="I9" s="8" t="n">
         <x:v>8</x:v>
       </x:c>
     </x:row>
@@ -1367,13 +1395,16 @@
       <x:c r="E10" s="8" t="str">
         <x:v>50% 38%</x:v>
       </x:c>
-      <x:c r="F10" s="8" t="n">
+      <x:c r="F10" s="8" t="str">
+        <x:v>https://pag.ae/81Zp4c6TK</x:v>
+      </x:c>
+      <x:c r="G10" s="8" t="n">
         <x:v>2000</x:v>
       </x:c>
-      <x:c r="G10" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="H10" s="8" t="n">
+      <x:c r="H10" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="I10" s="8" t="n">
         <x:v>9</x:v>
       </x:c>
     </x:row>
@@ -1393,13 +1424,16 @@
       <x:c r="E11" s="8" t="str">
         <x:v>50% 46%</x:v>
       </x:c>
-      <x:c r="F11" s="8" t="n">
+      <x:c r="F11" s="8" t="str">
+        <x:v>https://pag.ae/81Zp4LoX7</x:v>
+      </x:c>
+      <x:c r="G11" s="8" t="n">
         <x:v>5000</x:v>
       </x:c>
-      <x:c r="G11" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="H11" s="8" t="n">
+      <x:c r="H11" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="I11" s="8" t="n">
         <x:v>10</x:v>
       </x:c>
     </x:row>
@@ -1419,13 +1453,16 @@
       <x:c r="E12" s="8" t="str">
         <x:v>50% 50%</x:v>
       </x:c>
-      <x:c r="F12" s="8" t="n">
+      <x:c r="F12" s="8" t="str">
+        <x:v>https://pag.ae/81Zp59c14</x:v>
+      </x:c>
+      <x:c r="G12" s="8" t="n">
         <x:v>10000</x:v>
       </x:c>
-      <x:c r="G12" s="8" t="str">
-        <x:v>TRUE</x:v>
-      </x:c>
-      <x:c r="H12" s="8" t="n">
+      <x:c r="H12" s="8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="I12" s="8" t="n">
         <x:v>11</x:v>
       </x:c>
     </x:row>

</xml_diff>